<commit_message>
updated appendix A, B, C, D
</commit_message>
<xml_diff>
--- a/code/07_synthesis_results/environmental_data.xlsx
+++ b/code/07_synthesis_results/environmental_data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\41001583_faglig_utvikling_bernardo_dos_santos\07_projects\12_cumulative_impacts_mala\code\07_synthesis_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://svelantbruksuniversitet.sharepoint.com/sites/strim20192/Delade dokument/General/Malå/paper/text/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{617C20BF-D1F5-4685-A595-4B11F1DC1B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="187" documentId="8_{617C20BF-D1F5-4685-A595-4B11F1DC1B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15CD380E-BB9F-4BC0-AEE9-41FC08A651E3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F3714683-932F-4239-A00B-A5D8C4F777D1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F3714683-932F-4239-A00B-A5D8C4F777D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="57">
   <si>
     <t>Layer</t>
   </si>
@@ -44,6 +44,9 @@
     <t>Description</t>
   </si>
   <si>
+    <t>Image type</t>
+  </si>
+  <si>
     <t>Year</t>
   </si>
   <si>
@@ -59,59 +62,169 @@
     <t>Land use and land cover</t>
   </si>
   <si>
-    <t>Start of season (SOS) and end of season (EOS)</t>
+    <t>National Land Cover Database (NMD). Land cover map over Sweden with 25 thematic classes. Classified using Snetinel-2 satellite images and LIDAR data as well as existing national maps like soil maps, hydography, roads and buildings. The original classes are: 111 – Pine forest not on wetlands, 112 – Spruce forest not on wetlands, 113 – Mixed coniferous forest not on wetlands, 114 – Broadleaved forest not on wetlands, 115 – Mixed forest not on wetlands, 116 – Temporarily non-forest (clear-cuts etc.) not on wetlands, 121 – Pine forest on wetlands, 122 – Spruce forest on wetlands, 123 – Mixed coniferous forest on wetlands, 124 – Broadleaved forest on wetlands, 125 – Mixed forest on wetlands, 126 – Temporarily non-forest (clear-cuts etc.) on wetlands, 211 – Arable land, 212 – Grassland, 221 – Artificial surfaces, 231 – Bare rock and other areas with sparse vegetation, 241 – Open wetlands, 242 – Forested wetlands, 251 – Natural grasslands, 252 – Alpine heaths, 253 – Alpine meadows, 261 – Glaciers and permanent snow, 271 – Inland water, 272 – Marine water. The classes were re-classified as: deciduous forest (114, 124), coniferous forest (111, 112, 113, 115, 121, 122, 123), open areas (116, 211, 212, 231, 251, 252, 253), mires (125, 241, 242), and anthropogenic areas (221). Classes 261 and 272 were not present in the study area, and class 271 was removed because few GPS position were found within water.</t>
+  </si>
+  <si>
+    <t>Raster</t>
+  </si>
+  <si>
+    <t>10 m</t>
+  </si>
+  <si>
+    <t>https://www.naturvardsverket.se/en/services-and-permits/maps-and-map-services/national-land-cover-database/</t>
+  </si>
+  <si>
+    <t>Clear cuts</t>
+  </si>
+  <si>
+    <t>Final fellings data from the Forest Attribute Map (Digital Open Forest Data), consisting of polygons and corresponding year of cut. Clear cuts year was compared with the acquisition time of GPS positions and land use classes were updated for those positions when the acquisition time occurred after the clear cut year.</t>
+  </si>
+  <si>
+    <t>Vector</t>
+  </si>
+  <si>
+    <t>The Swedish Forest Agency</t>
+  </si>
+  <si>
+    <t>https://www.skogsstyrelsen.se/en/digital-open-forest-data/</t>
+  </si>
+  <si>
+    <t>Start of season (SOS), end of season (EOS), and instantaneous rate of green-up (IRG)</t>
+  </si>
+  <si>
+    <t>Derived from Normalized Difference Vegetation Index (NDVI) downloaded from Google Earth Engine (MOD13Q1.061 Terra Vegetation Indices 16-Day Global 250 m) using the R package phenofit (https://github.com/eco-hydro/phenofit).</t>
+  </si>
+  <si>
+    <t>250 m</t>
+  </si>
+  <si>
+    <t>Google Earth Engine</t>
+  </si>
+  <si>
+    <t>https://developers.google.com/earth-engine/datasets/catalog/MODIS_061_MOD13Q1</t>
   </si>
   <si>
     <t>Elevation</t>
   </si>
   <si>
+    <t>Terrain model of Sweden</t>
+  </si>
+  <si>
+    <t>Lantmäteriet (Swedish mapping, cadastral and land registration authority)</t>
+  </si>
+  <si>
+    <t>https://www.lantmateriet.se/en/geodata/our-products/product-list/elevation-model-download/</t>
+  </si>
+  <si>
     <t>Slope, aspect</t>
   </si>
   <si>
-    <t>TPI</t>
+    <t xml:space="preserve">Derived from elevation using the module r.slope.aspect in GRASS GIS 7.8. </t>
+  </si>
+  <si>
+    <t>Computed for this study</t>
+  </si>
+  <si>
+    <t>Derived data</t>
+  </si>
+  <si>
+    <t>Terrain position index (TPI)</t>
+  </si>
+  <si>
+    <t>Computed based on the elevation, with neighborhood sizes 150 m, 250 m, and 510 m. TPI was reclassified following  the approach from Weiss (2001) into six categories: valley, lower slope,  flat, middle slope, upper slope, ridge. Reference: Weiss, A.D., 2001. Topographic Position and Landforms Analysis. ESRI User Conference.</t>
   </si>
   <si>
     <t>Wind turbines</t>
   </si>
   <si>
-    <t>ZOI of wind turbines</t>
+    <t>Position for each wind turbine, not used directly in the analysis</t>
+  </si>
+  <si>
+    <t>County administrative boards and Swedish Energy Agency</t>
+  </si>
+  <si>
+    <t>https://ext-webbgis.lansstyrelsen.se/vbk/</t>
+  </si>
+  <si>
+    <t>Zone of influence (ZOI) of wind turbines</t>
+  </si>
+  <si>
+    <t>Either the density of wind turbines of and the decay-distance to the nearest wind turbine, computed at scales 100 m, 250 m, 500 m, 1 km, 2.5 km, 5 km, and 10 km. ZOIs were computed using an exponential distance decay shape using the oneimpact package in R (https://github.com/NINAnor/oneimpact/).</t>
   </si>
   <si>
     <t>Mines</t>
   </si>
   <si>
-    <t>ZOI of mine</t>
-  </si>
-  <si>
-    <t>Both density and nearest, computed at scales 100, …, 10km, using the oneimpact package etc</t>
+    <t>Active mining areas</t>
+  </si>
+  <si>
+    <t>The Geological Survey of Sweden (SGU)</t>
+  </si>
+  <si>
+    <t>https://apps.sgu.se/kartvisare/kartvisare-mineralrattigheter.html</t>
+  </si>
+  <si>
+    <t>Zone of influence (ZOI) of mine</t>
+  </si>
+  <si>
+    <t>Computed considering an exponential decay distance to the mine, with ZOI radius 100 m, 250 m, 500 m, 1 km, 2.5 km, 5 km, and 10 km. ZOIs were computed using the oneimpact package in R (https://github.com/NINAnor/oneimpact/).</t>
   </si>
   <si>
     <t>Public roads</t>
   </si>
   <si>
+    <t>Public (main) roads. Used to compute the (log) distance to the nearest feature, used in the statistical models.</t>
+  </si>
+  <si>
+    <t>https://www.lantmateriet.se/en/geodata/our-products/product-list/topography-10-download-vector/</t>
+  </si>
+  <si>
     <t>Private roads</t>
   </si>
   <si>
+    <t>Private roads (mostly private and forestry roads). Used to compute the (log) distance to the nearest feature as input for the statistical models.</t>
+  </si>
+  <si>
+    <t>Trails</t>
+  </si>
+  <si>
+    <t>Tourist trails. Used to compute the (log) distance to the nearest feature as input for the statistical models.</t>
+  </si>
+  <si>
     <t>Power lines</t>
   </si>
   <si>
-    <t>Trails</t>
+    <t>Power lines. Used to compute the (log) distance to the nearest feature as input for the statistical models.</t>
   </si>
   <si>
     <t>Houses</t>
   </si>
   <si>
-    <t>What else?</t>
+    <t>Houses and associated building. Used to compute the (log) distance to the nearest feature as input for the statistical models.</t>
+  </si>
+  <si>
+    <t>Swedish Environmental Protection Agency (Naturvårdsverket)</t>
+  </si>
+  <si>
+    <t>1 m, resampled to 10 m</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -134,13 +247,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -473,17 +589,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F56488C2-0863-486A-A85C-2F6DE3361B55}">
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="102" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="69.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -502,86 +619,610 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2">
+        <v>2018</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>2020</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>2022</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>2019</v>
+      </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9">
+        <v>2019</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12">
+        <v>2019</v>
+      </c>
+      <c r="F12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13">
+        <v>2019</v>
+      </c>
+      <c r="F13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="B14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14">
+        <v>2019</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15">
+        <v>2019</v>
+      </c>
+      <c r="F15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16">
+        <v>2019</v>
+      </c>
+      <c r="F16" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G8" r:id="rId1" xr:uid="{3E7E71D1-9707-4103-897B-51B23BDC6956}"/>
+    <hyperlink ref="G12" r:id="rId2" xr:uid="{671AB171-9204-455B-A984-D28DF12A0788}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{12BD6D96-6BE3-467B-A26B-3D3682165741}"/>
+    <hyperlink ref="G3" r:id="rId4" xr:uid="{858FF23B-82B3-4EE6-84C1-45CBBD9EF7FC}"/>
+    <hyperlink ref="G13" r:id="rId5" xr:uid="{34BD574C-38E3-428D-B017-20BA2D78F617}"/>
+    <hyperlink ref="G14" r:id="rId6" xr:uid="{80B267CC-6242-445D-ACF2-48247443536C}"/>
+    <hyperlink ref="G15" r:id="rId7" xr:uid="{DDC43206-E6B1-4BDE-8D4D-96F8B8CE0015}"/>
+    <hyperlink ref="G16" r:id="rId8" xr:uid="{4C4FD16B-395A-49EA-8A0F-7B9DFE5889AB}"/>
+    <hyperlink ref="G10" r:id="rId9" xr:uid="{87869219-BD91-467C-B5DB-96F0479D47FE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x010100F5ECF845D3105F4082E0E3E9915F18CB" ma:contentTypeVersion="18" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="252c1619c638012a058ce6de8241f0ad">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ab3444ca-12a4-4aff-9c00-912a6b9d0211" xmlns:ns3="8f7c5d63-507a-4e62-a899-e0e96f5526ce" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8ef5ce4c56262635dbbf8dcf706b54ed" ns2:_="" ns3:_="">
+    <xsd:import namespace="ab3444ca-12a4-4aff-9c00-912a6b9d0211"/>
+    <xsd:import namespace="8f7c5d63-507a-4e62-a899-e0e96f5526ce"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ab3444ca-12a4-4aff-9c00-912a6b9d0211" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="14" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="15" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="16" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Bildmarkeringar" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="357ce2f8-f89c-471c-b8ae-5f01d9449647" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="21" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8f7c5d63-507a-4e62-a899-e0e96f5526ce" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="18" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{e55fc425-1430-4dbb-a77d-1661064f952a}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="8f7c5d63-507a-4e62-a899-e0e96f5526ce">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Innehållstyp"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Rubrik"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8f7c5d63-507a-4e62-a899-e0e96f5526ce" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ab3444ca-12a4-4aff-9c00-912a6b9d0211">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BBC9CF1-CFE3-4224-943A-67B31AE1C327}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ab3444ca-12a4-4aff-9c00-912a6b9d0211"/>
+    <ds:schemaRef ds:uri="8f7c5d63-507a-4e62-a899-e0e96f5526ce"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E5EC724-8273-48FA-8C30-CC74F41BFD98}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8f7c5d63-507a-4e62-a899-e0e96f5526ce"/>
+    <ds:schemaRef ds:uri="ab3444ca-12a4-4aff-9c00-912a6b9d0211"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E5C72FE-1605-4A44-A985-0A2D14FD4DF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a3b5f071-0e49-47a0-a40e-9b7c9c4d647e}" enabled="0" method="" siteId="{a3b5f071-0e49-47a0-a40e-9b7c9c4d647e}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>